<commit_message>
Update local project state
</commit_message>
<xml_diff>
--- a/output_plant/stomata_Intermediate_beerling_2009.xlsx
+++ b/output_plant/stomata_Intermediate_beerling_2009.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="262">
   <si>
     <t>eDab</t>
   </si>
@@ -603,34 +603,175 @@
     <t xml:space="preserve"/>
   </si>
   <si>
+    <t xml:space="preserve">LJH 7659 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.2475/09.2009.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stomata-si_beerling_2009_p1.0.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harper and Giulivi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dustin.t.harper@utah.edu; claudiag@ldeo.columbia.edu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biostratigraphy (early Puercan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ginkgoaceae / Ginkgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ginkgoaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ginkgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original CO2 estimates made by Beerling et al. (2002 PNAS 99: 7836-7840 doi:10.1073 pnas.122573099) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; Milligan et al. (2019 Geophysical Research Letters doi:10.1029/2018GL081215) used the same cuticles to estimate CO2 with the Franks leaf-gas-exchange proxy; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LJH 7423 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original CO2 estimates made by Beerling et al. (2002 PNAS 99: 7836-7840 doi:10.1073 pnas.122573099) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMNH 2360 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">radiometric dating (Raynolds et al., 2001, p. 21; see Royer 2003 for citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basilika site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biostratigraphy (early Paleocene)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMNH 2644 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biostratigraphy (Torrejonian-Tiffanian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original CO2 estimates made by Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burbank site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biostratigraphy (middle Tiffanian, Ti-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Original CO2 estimates made by Royer et al. (2001 Science 292: 2310-2313 doi:10.1126/science.292.5525.2310) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joffre Bridge site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 0025 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LJH 7132 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 993 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.7 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 992 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 991 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LJH 72141-1 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9155 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9411 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9434 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9715 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 Myrs before the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9050 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9936 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 8612 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Considered to be from within the PETM by Jolley et al. (2002 Geology 30: 7-10 doi:10.1130/0091-7613(2002)030&lt;0007:PTSMEF&gt;2.0.CO;2); this was subsequently sharply disputed (see May 2003 issue of Geology); consequently, no age uncertainties are given here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9812 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 Myrs after the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW 9915 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4 Myrs after the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW LB site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3 Myrs after the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLW H site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7 Myrs after the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LJH 9915 site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8 Myrs after the PETM (Age Model 2 in Wing et al., 2000, which uses measured sections, biostratigraphy, the PETM carbon isotope excursion, and one Ar/Ar radiometric date; see Royer 2003 for details and for Wing citation)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juliaetta site (P6)</t>
   </si>
   <si>
-    <t xml:space="preserve">10.2475/09.2009.01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ncei.noaa.gov/pub/data/paleo/climate_forcing/trace_gases/Paleo-pCO2/stomata-si_beerling_2009.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harper and Giulivi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dustin.t.harper@utah.edu; claudiag@ldeo.columbia.edu</t>
-  </si>
-  <si>
     <t xml:space="preserve">radiometric constraints (Reidel &amp; Fecht, 1987; 10.1130/0016-7606(1987)98&lt;664:thfeos&gt;2.0.co;2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ginkgoaceae / Ginkgo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ginkgoaceae</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ginkgo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Original CO2 estimates made by Royer et al. (2001 Science 292: 2310-2313 doi:10.1126/science.292.5525.2310) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
   </si>
   <si>
     <t xml:space="preserve">Clarkia site (P33a)</t>
@@ -649,7 +790,7 @@
     <t xml:space="preserve">Metasequoia</t>
   </si>
   <si>
-    <t xml:space="preserve">Original CO2 estimates made by Royer et al. (2001 Science 292: 2310-2313 doi:10.1126/science.292.5525.2310) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; Original CO2 estimates made by Royer et al. (2001 Science 292: 2310-2313 doi:10.1126/science.292.5525.2310) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; pos CO2 uncertainty is actually unbounded but has been set to 2000 ppm for plotting purposes only; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
+    <t xml:space="preserve">Original CO2 estimates made by Royer et al. (2001 Science 292: 2310-2313 doi:10.1126/science.292.5525.2310) and Royer (2003 GSA Special Paper 369: 79-93 doi:10.1130/0-8137-2369-8.79); revised by Beerling et al. (2009) using a more robust error propagation routine; pos CO2 uncertainty is actually unbounded but has been set to 2000 ppm for plotting purposes only; SD: fields-of-view were partly comprised of non-stomatal-bearing areas (for example, over top major veins); the field-of-view fraction that was usable was not measured; as such, the measured stomatal densities are not particularly useful.</t>
   </si>
   <si>
     <t xml:space="preserve">Clarkia site (P33b)</t>
@@ -1976,20 +2117,20 @@
         <v>200</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>46.52</v>
+        <v>44.95</v>
       </c>
       <c r="G5" s="20" t="n">
-        <v>-116.75</v>
+        <v>-108.87</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>16.5</v>
+        <v>65.4</v>
       </c>
       <c r="I5" s="23"/>
       <c r="J5" s="23" t="n">
-        <v>15</v>
+        <v>64.8</v>
       </c>
       <c r="K5" s="23" t="n">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>201</v>
@@ -2071,32 +2212,32 @@
         <v>200</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>46.99</v>
+        <v>45.07</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>-116.27</v>
+        <v>-108.85</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>15.78</v>
+        <v>65.4</v>
       </c>
       <c r="I6" s="23"/>
       <c r="J6" s="23" t="n">
-        <v>15.741</v>
+        <v>64.8</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>15.819</v>
+        <v>66</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="P6" s="26"/>
       <c r="Q6" s="26"/>
@@ -2146,12 +2287,12 @@
       <c r="BI6" s="1"/>
       <c r="BJ6" s="1"/>
       <c r="BK6" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>197</v>
@@ -2166,32 +2307,30 @@
         <v>200</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>46.99</v>
-      </c>
-      <c r="G7" s="25" t="n">
-        <v>-116.27</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="G7" s="25"/>
       <c r="H7" s="23" t="n">
-        <v>15.78</v>
+        <v>64.1</v>
       </c>
       <c r="I7" s="23"/>
       <c r="J7" s="23" t="n">
-        <v>15.741</v>
+        <v>63.9</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>15.819</v>
+        <v>64.3</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
@@ -2241,12 +2380,12 @@
       <c r="BI7" s="1"/>
       <c r="BJ7" s="1"/>
       <c r="BK7" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>197</v>
@@ -2261,32 +2400,30 @@
         <v>200</v>
       </c>
       <c r="F8" s="25" t="n">
-        <v>47.03</v>
-      </c>
-      <c r="G8" s="25" t="n">
-        <v>-116.34</v>
-      </c>
+        <v>77.5</v>
+      </c>
+      <c r="G8" s="25"/>
       <c r="H8" s="23" t="n">
-        <v>15.78</v>
+        <v>63.8</v>
       </c>
       <c r="I8" s="23"/>
       <c r="J8" s="23" t="n">
-        <v>15.741</v>
+        <v>61.6</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>15.819</v>
+        <v>66</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="P8" s="26"/>
       <c r="Q8" s="26"/>
@@ -2336,33 +2473,63 @@
       <c r="BI8" s="1"/>
       <c r="BJ8" s="1"/>
       <c r="BK8" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="25"/>
+      <c r="A9" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>42.5</v>
+      </c>
       <c r="G9" s="25"/>
-      <c r="H9" s="23"/>
+      <c r="H9" s="23" t="n">
+        <v>61.1</v>
+      </c>
       <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
+      <c r="J9" s="23" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P9" s="26"/>
       <c r="Q9" s="26"/>
+      <c r="R9"/>
       <c r="S9" s="24"/>
       <c r="T9" s="24"/>
+      <c r="U9"/>
       <c r="V9" s="26"/>
       <c r="W9" s="26"/>
+      <c r="X9"/>
       <c r="Y9" s="24"/>
       <c r="Z9" s="24"/>
+      <c r="AA9"/>
       <c r="AB9" s="24"/>
       <c r="AC9" s="24"/>
       <c r="AD9" s="1"/>
@@ -2371,6 +2538,7 @@
       <c r="AG9" s="1"/>
       <c r="AH9" s="25"/>
       <c r="AI9" s="25"/>
+      <c r="AJ9"/>
       <c r="AK9" s="1"/>
       <c r="AL9" s="1"/>
       <c r="AM9" s="1"/>
@@ -2397,32 +2565,64 @@
       <c r="BH9" s="1"/>
       <c r="BI9" s="1"/>
       <c r="BJ9" s="1"/>
-      <c r="BK9" s="1"/>
+      <c r="BK9" s="1" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="25"/>
+      <c r="A10" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>52.25</v>
+      </c>
       <c r="G10" s="25"/>
-      <c r="H10" s="23"/>
+      <c r="H10" s="23" t="n">
+        <v>59.9</v>
+      </c>
       <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="J10" s="23" t="n">
+        <v>59</v>
+      </c>
+      <c r="K10" s="23" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P10" s="26"/>
       <c r="Q10" s="26"/>
+      <c r="R10"/>
       <c r="S10" s="24"/>
       <c r="T10" s="24"/>
+      <c r="U10"/>
       <c r="V10" s="26"/>
       <c r="W10" s="26"/>
+      <c r="X10"/>
       <c r="Y10" s="24"/>
       <c r="Z10" s="24"/>
+      <c r="AA10"/>
       <c r="AB10" s="24"/>
       <c r="AC10" s="24"/>
       <c r="AD10" s="1"/>
@@ -2431,6 +2631,7 @@
       <c r="AG10" s="1"/>
       <c r="AH10" s="25"/>
       <c r="AI10" s="25"/>
+      <c r="AJ10"/>
       <c r="AK10" s="1"/>
       <c r="AL10" s="1"/>
       <c r="AM10" s="1"/>
@@ -2457,32 +2658,64 @@
       <c r="BH10" s="1"/>
       <c r="BI10" s="1"/>
       <c r="BJ10" s="1"/>
-      <c r="BK10" s="1"/>
+      <c r="BK10" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="25"/>
+      <c r="A11" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>52.25</v>
+      </c>
       <c r="G11" s="25"/>
-      <c r="H11" s="23"/>
+      <c r="H11" s="23" t="n">
+        <v>59.9</v>
+      </c>
       <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
+      <c r="J11" s="23" t="n">
+        <v>59</v>
+      </c>
+      <c r="K11" s="23" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P11" s="26"/>
       <c r="Q11" s="26"/>
+      <c r="R11"/>
       <c r="S11" s="24"/>
       <c r="T11" s="24"/>
+      <c r="U11"/>
       <c r="V11" s="26"/>
       <c r="W11" s="26"/>
+      <c r="X11"/>
       <c r="Y11" s="24"/>
       <c r="Z11" s="24"/>
+      <c r="AA11"/>
       <c r="AB11" s="24"/>
       <c r="AC11" s="24"/>
       <c r="AD11" s="1"/>
@@ -2491,6 +2724,7 @@
       <c r="AG11" s="1"/>
       <c r="AH11" s="25"/>
       <c r="AI11" s="25"/>
+      <c r="AJ11"/>
       <c r="AK11" s="1"/>
       <c r="AL11" s="1"/>
       <c r="AM11" s="1"/>
@@ -2517,32 +2751,66 @@
       <c r="BH11" s="1"/>
       <c r="BI11" s="1"/>
       <c r="BJ11" s="1"/>
-      <c r="BK11" s="1"/>
+      <c r="BK11" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="23"/>
+      <c r="A12" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>44.86</v>
+      </c>
+      <c r="G12" s="25" t="n">
+        <v>-108.88</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <v>58.1</v>
+      </c>
       <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
+      <c r="J12" s="23" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="K12" s="23" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P12" s="26"/>
       <c r="Q12" s="26"/>
+      <c r="R12"/>
       <c r="S12" s="24"/>
       <c r="T12" s="24"/>
+      <c r="U12"/>
       <c r="V12" s="26"/>
       <c r="W12" s="26"/>
+      <c r="X12"/>
       <c r="Y12" s="24"/>
       <c r="Z12" s="24"/>
+      <c r="AA12"/>
       <c r="AB12" s="24"/>
       <c r="AC12" s="24"/>
       <c r="AD12" s="1"/>
@@ -2551,6 +2819,7 @@
       <c r="AG12" s="1"/>
       <c r="AH12" s="25"/>
       <c r="AI12" s="25"/>
+      <c r="AJ12"/>
       <c r="AK12" s="1"/>
       <c r="AL12" s="1"/>
       <c r="AM12" s="1"/>
@@ -2577,32 +2846,66 @@
       <c r="BH12" s="1"/>
       <c r="BI12" s="1"/>
       <c r="BJ12" s="1"/>
-      <c r="BK12" s="1"/>
+      <c r="BK12" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="23"/>
+      <c r="A13" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>45.03</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>-109.08</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <v>57.2</v>
+      </c>
       <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
+      <c r="J13" s="23" t="n">
+        <v>57</v>
+      </c>
+      <c r="K13" s="23" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P13" s="26"/>
       <c r="Q13" s="26"/>
+      <c r="R13"/>
       <c r="S13" s="24"/>
       <c r="T13" s="24"/>
+      <c r="U13"/>
       <c r="V13" s="26"/>
       <c r="W13" s="26"/>
+      <c r="X13"/>
       <c r="Y13" s="24"/>
       <c r="Z13" s="24"/>
+      <c r="AA13"/>
       <c r="AB13" s="24"/>
       <c r="AC13" s="24"/>
       <c r="AD13" s="1"/>
@@ -2611,6 +2914,7 @@
       <c r="AG13" s="1"/>
       <c r="AH13" s="25"/>
       <c r="AI13" s="25"/>
+      <c r="AJ13"/>
       <c r="AK13" s="1"/>
       <c r="AL13" s="1"/>
       <c r="AM13" s="1"/>
@@ -2637,32 +2941,64 @@
       <c r="BH13" s="1"/>
       <c r="BI13" s="1"/>
       <c r="BJ13" s="1"/>
-      <c r="BK13" s="1"/>
+      <c r="BK13" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="25"/>
+      <c r="A14" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <v>44.8</v>
+      </c>
       <c r="G14" s="25"/>
-      <c r="H14" s="23"/>
+      <c r="H14" s="23" t="n">
+        <v>56.7</v>
+      </c>
       <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
+      <c r="J14" s="23" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="K14" s="23" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="P14" s="26"/>
       <c r="Q14" s="26"/>
+      <c r="R14"/>
       <c r="S14" s="24"/>
       <c r="T14" s="24"/>
+      <c r="U14"/>
       <c r="V14" s="26"/>
       <c r="W14" s="26"/>
+      <c r="X14"/>
       <c r="Y14" s="24"/>
       <c r="Z14" s="24"/>
+      <c r="AA14"/>
       <c r="AB14" s="24"/>
       <c r="AC14" s="24"/>
       <c r="AD14" s="1"/>
@@ -2671,6 +3007,7 @@
       <c r="AG14" s="1"/>
       <c r="AH14" s="25"/>
       <c r="AI14" s="25"/>
+      <c r="AJ14"/>
       <c r="AK14" s="1"/>
       <c r="AL14" s="1"/>
       <c r="AM14" s="1"/>
@@ -2697,147 +3034,1885 @@
       <c r="BH14" s="1"/>
       <c r="BI14" s="1"/>
       <c r="BJ14" s="1"/>
-      <c r="BK14" s="1"/>
+      <c r="BK14" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="15">
-      <c r="H15" s="23"/>
+      <c r="A15" t="s">
+        <v>225</v>
+      </c>
+      <c r="B15" t="s">
+        <v>197</v>
+      </c>
+      <c r="C15" t="s">
+        <v>198</v>
+      </c>
+      <c r="D15" t="s">
+        <v>199</v>
+      </c>
+      <c r="E15" t="s">
+        <v>200</v>
+      </c>
+      <c r="F15" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G15"/>
+      <c r="H15" s="23" t="n">
+        <v>56.7</v>
+      </c>
       <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="BK15" s="1"/>
+      <c r="J15" s="23" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="K15" s="23" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="L15" t="s">
+        <v>224</v>
+      </c>
+      <c r="M15" t="s">
+        <v>202</v>
+      </c>
+      <c r="N15" t="s">
+        <v>203</v>
+      </c>
+      <c r="O15" t="s">
+        <v>204</v>
+      </c>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
+      <c r="W15"/>
+      <c r="X15"/>
+      <c r="Y15"/>
+      <c r="Z15"/>
+      <c r="AA15"/>
+      <c r="AB15"/>
+      <c r="AC15"/>
+      <c r="AD15"/>
+      <c r="AE15"/>
+      <c r="AF15"/>
+      <c r="AG15"/>
+      <c r="AH15"/>
+      <c r="AI15"/>
+      <c r="AJ15"/>
+      <c r="AK15"/>
+      <c r="AL15"/>
+      <c r="AM15"/>
+      <c r="AN15"/>
+      <c r="AO15"/>
+      <c r="AP15"/>
+      <c r="AQ15"/>
+      <c r="AR15"/>
+      <c r="AS15"/>
+      <c r="AT15"/>
+      <c r="AU15"/>
+      <c r="AV15"/>
+      <c r="AW15"/>
+      <c r="AX15"/>
+      <c r="AY15"/>
+      <c r="AZ15"/>
+      <c r="BA15"/>
+      <c r="BB15"/>
+      <c r="BC15"/>
+      <c r="BD15"/>
+      <c r="BE15"/>
+      <c r="BF15"/>
+      <c r="BG15"/>
+      <c r="BH15"/>
+      <c r="BI15"/>
+      <c r="BJ15"/>
+      <c r="BK15" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="16">
-      <c r="H16" s="23"/>
+      <c r="A16" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D16" t="s">
+        <v>199</v>
+      </c>
+      <c r="E16" t="s">
+        <v>200</v>
+      </c>
+      <c r="F16" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G16"/>
+      <c r="H16" s="23" t="n">
+        <v>56.7</v>
+      </c>
       <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="BK16" s="1"/>
+      <c r="J16" s="23" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="K16" s="23" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="L16" t="s">
+        <v>224</v>
+      </c>
+      <c r="M16" t="s">
+        <v>202</v>
+      </c>
+      <c r="N16" t="s">
+        <v>203</v>
+      </c>
+      <c r="O16" t="s">
+        <v>204</v>
+      </c>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
+      <c r="W16"/>
+      <c r="X16"/>
+      <c r="Y16"/>
+      <c r="Z16"/>
+      <c r="AA16"/>
+      <c r="AB16"/>
+      <c r="AC16"/>
+      <c r="AD16"/>
+      <c r="AE16"/>
+      <c r="AF16"/>
+      <c r="AG16"/>
+      <c r="AH16"/>
+      <c r="AI16"/>
+      <c r="AJ16"/>
+      <c r="AK16"/>
+      <c r="AL16"/>
+      <c r="AM16"/>
+      <c r="AN16"/>
+      <c r="AO16"/>
+      <c r="AP16"/>
+      <c r="AQ16"/>
+      <c r="AR16"/>
+      <c r="AS16"/>
+      <c r="AT16"/>
+      <c r="AU16"/>
+      <c r="AV16"/>
+      <c r="AW16"/>
+      <c r="AX16"/>
+      <c r="AY16"/>
+      <c r="AZ16"/>
+      <c r="BA16"/>
+      <c r="BB16"/>
+      <c r="BC16"/>
+      <c r="BD16"/>
+      <c r="BE16"/>
+      <c r="BF16"/>
+      <c r="BG16"/>
+      <c r="BH16"/>
+      <c r="BI16"/>
+      <c r="BJ16"/>
+      <c r="BK16" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="17">
-      <c r="H17" s="23"/>
+      <c r="A17" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" t="s">
+        <v>197</v>
+      </c>
+      <c r="C17" t="s">
+        <v>198</v>
+      </c>
+      <c r="D17" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" t="s">
+        <v>200</v>
+      </c>
+      <c r="F17" t="n">
+        <v>44.73</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-108.68</v>
+      </c>
+      <c r="H17" s="23" t="n">
+        <v>56.6</v>
+      </c>
       <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="BK17" s="1"/>
+      <c r="J17" s="23" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="K17" s="23" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="L17" t="s">
+        <v>228</v>
+      </c>
+      <c r="M17" t="s">
+        <v>202</v>
+      </c>
+      <c r="N17" t="s">
+        <v>203</v>
+      </c>
+      <c r="O17" t="s">
+        <v>204</v>
+      </c>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
+      <c r="W17"/>
+      <c r="X17"/>
+      <c r="Y17"/>
+      <c r="Z17"/>
+      <c r="AA17"/>
+      <c r="AB17"/>
+      <c r="AC17"/>
+      <c r="AD17"/>
+      <c r="AE17"/>
+      <c r="AF17"/>
+      <c r="AG17"/>
+      <c r="AH17"/>
+      <c r="AI17"/>
+      <c r="AJ17"/>
+      <c r="AK17"/>
+      <c r="AL17"/>
+      <c r="AM17"/>
+      <c r="AN17"/>
+      <c r="AO17"/>
+      <c r="AP17"/>
+      <c r="AQ17"/>
+      <c r="AR17"/>
+      <c r="AS17"/>
+      <c r="AT17"/>
+      <c r="AU17"/>
+      <c r="AV17"/>
+      <c r="AW17"/>
+      <c r="AX17"/>
+      <c r="AY17"/>
+      <c r="AZ17"/>
+      <c r="BA17"/>
+      <c r="BB17"/>
+      <c r="BC17"/>
+      <c r="BD17"/>
+      <c r="BE17"/>
+      <c r="BF17"/>
+      <c r="BG17"/>
+      <c r="BH17"/>
+      <c r="BI17"/>
+      <c r="BJ17"/>
+      <c r="BK17" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="18">
-      <c r="H18" s="23"/>
+      <c r="A18" t="s">
+        <v>229</v>
+      </c>
+      <c r="B18" t="s">
+        <v>197</v>
+      </c>
+      <c r="C18" t="s">
+        <v>198</v>
+      </c>
+      <c r="D18" t="s">
+        <v>199</v>
+      </c>
+      <c r="E18" t="s">
+        <v>200</v>
+      </c>
+      <c r="F18" t="n">
+        <v>44.05</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-107.77</v>
+      </c>
+      <c r="H18" s="23" t="n">
+        <v>56.5</v>
+      </c>
       <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="BK18" s="1"/>
+      <c r="J18" s="23" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="K18" s="23" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="L18" t="s">
+        <v>230</v>
+      </c>
+      <c r="M18" t="s">
+        <v>202</v>
+      </c>
+      <c r="N18" t="s">
+        <v>203</v>
+      </c>
+      <c r="O18" t="s">
+        <v>204</v>
+      </c>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+      <c r="W18"/>
+      <c r="X18"/>
+      <c r="Y18"/>
+      <c r="Z18"/>
+      <c r="AA18"/>
+      <c r="AB18"/>
+      <c r="AC18"/>
+      <c r="AD18"/>
+      <c r="AE18"/>
+      <c r="AF18"/>
+      <c r="AG18"/>
+      <c r="AH18"/>
+      <c r="AI18"/>
+      <c r="AJ18"/>
+      <c r="AK18"/>
+      <c r="AL18"/>
+      <c r="AM18"/>
+      <c r="AN18"/>
+      <c r="AO18"/>
+      <c r="AP18"/>
+      <c r="AQ18"/>
+      <c r="AR18"/>
+      <c r="AS18"/>
+      <c r="AT18"/>
+      <c r="AU18"/>
+      <c r="AV18"/>
+      <c r="AW18"/>
+      <c r="AX18"/>
+      <c r="AY18"/>
+      <c r="AZ18"/>
+      <c r="BA18"/>
+      <c r="BB18"/>
+      <c r="BC18"/>
+      <c r="BD18"/>
+      <c r="BE18"/>
+      <c r="BF18"/>
+      <c r="BG18"/>
+      <c r="BH18"/>
+      <c r="BI18"/>
+      <c r="BJ18"/>
+      <c r="BK18" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="19">
-      <c r="H19" s="23"/>
+      <c r="A19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C19" t="s">
+        <v>198</v>
+      </c>
+      <c r="D19" t="s">
+        <v>199</v>
+      </c>
+      <c r="E19" t="s">
+        <v>200</v>
+      </c>
+      <c r="F19" t="n">
+        <v>43.95</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-107.56</v>
+      </c>
+      <c r="H19" s="23" t="n">
+        <v>56.4</v>
+      </c>
       <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="BK19" s="1"/>
+      <c r="J19" s="23" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="K19" s="23" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="L19" t="s">
+        <v>232</v>
+      </c>
+      <c r="M19" t="s">
+        <v>202</v>
+      </c>
+      <c r="N19" t="s">
+        <v>203</v>
+      </c>
+      <c r="O19" t="s">
+        <v>204</v>
+      </c>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
+      <c r="W19"/>
+      <c r="X19"/>
+      <c r="Y19"/>
+      <c r="Z19"/>
+      <c r="AA19"/>
+      <c r="AB19"/>
+      <c r="AC19"/>
+      <c r="AD19"/>
+      <c r="AE19"/>
+      <c r="AF19"/>
+      <c r="AG19"/>
+      <c r="AH19"/>
+      <c r="AI19"/>
+      <c r="AJ19"/>
+      <c r="AK19"/>
+      <c r="AL19"/>
+      <c r="AM19"/>
+      <c r="AN19"/>
+      <c r="AO19"/>
+      <c r="AP19"/>
+      <c r="AQ19"/>
+      <c r="AR19"/>
+      <c r="AS19"/>
+      <c r="AT19"/>
+      <c r="AU19"/>
+      <c r="AV19"/>
+      <c r="AW19"/>
+      <c r="AX19"/>
+      <c r="AY19"/>
+      <c r="AZ19"/>
+      <c r="BA19"/>
+      <c r="BB19"/>
+      <c r="BC19"/>
+      <c r="BD19"/>
+      <c r="BE19"/>
+      <c r="BF19"/>
+      <c r="BG19"/>
+      <c r="BH19"/>
+      <c r="BI19"/>
+      <c r="BJ19"/>
+      <c r="BK19" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="20">
-      <c r="H20" s="23"/>
+      <c r="A20" t="s">
+        <v>233</v>
+      </c>
+      <c r="B20" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" t="s">
+        <v>198</v>
+      </c>
+      <c r="D20" t="s">
+        <v>199</v>
+      </c>
+      <c r="E20" t="s">
+        <v>200</v>
+      </c>
+      <c r="F20" t="n">
+        <v>44.16</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-107.85</v>
+      </c>
+      <c r="H20" s="23" t="n">
+        <v>56.2</v>
+      </c>
       <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="BK20" s="1"/>
+      <c r="J20" s="23" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="K20" s="23" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="L20" t="s">
+        <v>234</v>
+      </c>
+      <c r="M20" t="s">
+        <v>202</v>
+      </c>
+      <c r="N20" t="s">
+        <v>203</v>
+      </c>
+      <c r="O20" t="s">
+        <v>204</v>
+      </c>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+      <c r="AR20"/>
+      <c r="AS20"/>
+      <c r="AT20"/>
+      <c r="AU20"/>
+      <c r="AV20"/>
+      <c r="AW20"/>
+      <c r="AX20"/>
+      <c r="AY20"/>
+      <c r="AZ20"/>
+      <c r="BA20"/>
+      <c r="BB20"/>
+      <c r="BC20"/>
+      <c r="BD20"/>
+      <c r="BE20"/>
+      <c r="BF20"/>
+      <c r="BG20"/>
+      <c r="BH20"/>
+      <c r="BI20"/>
+      <c r="BJ20"/>
+      <c r="BK20" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="21">
-      <c r="H21" s="23"/>
+      <c r="A21" t="s">
+        <v>235</v>
+      </c>
+      <c r="B21" t="s">
+        <v>197</v>
+      </c>
+      <c r="C21" t="s">
+        <v>198</v>
+      </c>
+      <c r="D21" t="s">
+        <v>199</v>
+      </c>
+      <c r="E21" t="s">
+        <v>200</v>
+      </c>
+      <c r="F21" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G21"/>
+      <c r="H21" s="23" t="n">
+        <v>56.1</v>
+      </c>
       <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="BK21" s="1"/>
+      <c r="J21" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="K21" s="23" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="L21" t="s">
+        <v>236</v>
+      </c>
+      <c r="M21" t="s">
+        <v>202</v>
+      </c>
+      <c r="N21" t="s">
+        <v>203</v>
+      </c>
+      <c r="O21" t="s">
+        <v>204</v>
+      </c>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
+      <c r="W21"/>
+      <c r="X21"/>
+      <c r="Y21"/>
+      <c r="Z21"/>
+      <c r="AA21"/>
+      <c r="AB21"/>
+      <c r="AC21"/>
+      <c r="AD21"/>
+      <c r="AE21"/>
+      <c r="AF21"/>
+      <c r="AG21"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
+      <c r="AJ21"/>
+      <c r="AK21"/>
+      <c r="AL21"/>
+      <c r="AM21"/>
+      <c r="AN21"/>
+      <c r="AO21"/>
+      <c r="AP21"/>
+      <c r="AQ21"/>
+      <c r="AR21"/>
+      <c r="AS21"/>
+      <c r="AT21"/>
+      <c r="AU21"/>
+      <c r="AV21"/>
+      <c r="AW21"/>
+      <c r="AX21"/>
+      <c r="AY21"/>
+      <c r="AZ21"/>
+      <c r="BA21"/>
+      <c r="BB21"/>
+      <c r="BC21"/>
+      <c r="BD21"/>
+      <c r="BE21"/>
+      <c r="BF21"/>
+      <c r="BG21"/>
+      <c r="BH21"/>
+      <c r="BI21"/>
+      <c r="BJ21"/>
+      <c r="BK21" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="22">
-      <c r="H22" s="23"/>
+      <c r="A22" t="s">
+        <v>237</v>
+      </c>
+      <c r="B22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C22" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" t="s">
+        <v>199</v>
+      </c>
+      <c r="E22" t="s">
+        <v>200</v>
+      </c>
+      <c r="F22" t="n">
+        <v>43.95</v>
+      </c>
+      <c r="G22"/>
+      <c r="H22" s="23" t="n">
+        <v>56.1</v>
+      </c>
       <c r="I22" s="23"/>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="BK22" s="1"/>
+      <c r="J22" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="K22" s="23" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="L22" t="s">
+        <v>236</v>
+      </c>
+      <c r="M22" t="s">
+        <v>202</v>
+      </c>
+      <c r="N22" t="s">
+        <v>203</v>
+      </c>
+      <c r="O22" t="s">
+        <v>204</v>
+      </c>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22"/>
+      <c r="V22"/>
+      <c r="W22"/>
+      <c r="X22"/>
+      <c r="Y22"/>
+      <c r="Z22"/>
+      <c r="AA22"/>
+      <c r="AB22"/>
+      <c r="AC22"/>
+      <c r="AD22"/>
+      <c r="AE22"/>
+      <c r="AF22"/>
+      <c r="AG22"/>
+      <c r="AH22"/>
+      <c r="AI22"/>
+      <c r="AJ22"/>
+      <c r="AK22"/>
+      <c r="AL22"/>
+      <c r="AM22"/>
+      <c r="AN22"/>
+      <c r="AO22"/>
+      <c r="AP22"/>
+      <c r="AQ22"/>
+      <c r="AR22"/>
+      <c r="AS22"/>
+      <c r="AT22"/>
+      <c r="AU22"/>
+      <c r="AV22"/>
+      <c r="AW22"/>
+      <c r="AX22"/>
+      <c r="AY22"/>
+      <c r="AZ22"/>
+      <c r="BA22"/>
+      <c r="BB22"/>
+      <c r="BC22"/>
+      <c r="BD22"/>
+      <c r="BE22"/>
+      <c r="BF22"/>
+      <c r="BG22"/>
+      <c r="BH22"/>
+      <c r="BI22"/>
+      <c r="BJ22"/>
+      <c r="BK22" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="23">
-      <c r="H23" s="23"/>
+      <c r="A23" t="s">
+        <v>238</v>
+      </c>
+      <c r="B23" t="s">
+        <v>197</v>
+      </c>
+      <c r="C23" t="s">
+        <v>198</v>
+      </c>
+      <c r="D23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E23" t="s">
+        <v>200</v>
+      </c>
+      <c r="F23" t="n">
+        <v>43.95</v>
+      </c>
+      <c r="G23"/>
+      <c r="H23" s="23" t="n">
+        <v>56.1</v>
+      </c>
       <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="BK23" s="1"/>
+      <c r="J23" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="K23" s="23" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="L23" t="s">
+        <v>236</v>
+      </c>
+      <c r="M23" t="s">
+        <v>202</v>
+      </c>
+      <c r="N23" t="s">
+        <v>203</v>
+      </c>
+      <c r="O23" t="s">
+        <v>204</v>
+      </c>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+      <c r="AR23"/>
+      <c r="AS23"/>
+      <c r="AT23"/>
+      <c r="AU23"/>
+      <c r="AV23"/>
+      <c r="AW23"/>
+      <c r="AX23"/>
+      <c r="AY23"/>
+      <c r="AZ23"/>
+      <c r="BA23"/>
+      <c r="BB23"/>
+      <c r="BC23"/>
+      <c r="BD23"/>
+      <c r="BE23"/>
+      <c r="BF23"/>
+      <c r="BG23"/>
+      <c r="BH23"/>
+      <c r="BI23"/>
+      <c r="BJ23"/>
+      <c r="BK23" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="24">
-      <c r="H24" s="23"/>
+      <c r="A24" t="s">
+        <v>239</v>
+      </c>
+      <c r="B24" t="s">
+        <v>197</v>
+      </c>
+      <c r="C24" t="s">
+        <v>198</v>
+      </c>
+      <c r="D24" t="s">
+        <v>199</v>
+      </c>
+      <c r="E24" t="s">
+        <v>200</v>
+      </c>
+      <c r="F24" t="n">
+        <v>44.15</v>
+      </c>
+      <c r="G24"/>
+      <c r="H24" s="23" t="n">
+        <v>56.1</v>
+      </c>
       <c r="I24" s="23"/>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="BK24" s="1"/>
+      <c r="J24" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="K24" s="23" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="L24" t="s">
+        <v>236</v>
+      </c>
+      <c r="M24" t="s">
+        <v>202</v>
+      </c>
+      <c r="N24" t="s">
+        <v>203</v>
+      </c>
+      <c r="O24" t="s">
+        <v>204</v>
+      </c>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
+      <c r="W24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+      <c r="Z24"/>
+      <c r="AA24"/>
+      <c r="AB24"/>
+      <c r="AC24"/>
+      <c r="AD24"/>
+      <c r="AE24"/>
+      <c r="AF24"/>
+      <c r="AG24"/>
+      <c r="AH24"/>
+      <c r="AI24"/>
+      <c r="AJ24"/>
+      <c r="AK24"/>
+      <c r="AL24"/>
+      <c r="AM24"/>
+      <c r="AN24"/>
+      <c r="AO24"/>
+      <c r="AP24"/>
+      <c r="AQ24"/>
+      <c r="AR24"/>
+      <c r="AS24"/>
+      <c r="AT24"/>
+      <c r="AU24"/>
+      <c r="AV24"/>
+      <c r="AW24"/>
+      <c r="AX24"/>
+      <c r="AY24"/>
+      <c r="AZ24"/>
+      <c r="BA24"/>
+      <c r="BB24"/>
+      <c r="BC24"/>
+      <c r="BD24"/>
+      <c r="BE24"/>
+      <c r="BF24"/>
+      <c r="BG24"/>
+      <c r="BH24"/>
+      <c r="BI24"/>
+      <c r="BJ24"/>
+      <c r="BK24" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="25">
-      <c r="H25" s="23"/>
+      <c r="A25"/>
+      <c r="B25" t="s">
+        <v>197</v>
+      </c>
+      <c r="C25" t="s">
+        <v>198</v>
+      </c>
+      <c r="D25" t="s">
+        <v>199</v>
+      </c>
+      <c r="E25" t="s">
+        <v>200</v>
+      </c>
+      <c r="F25" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <v>56</v>
+      </c>
       <c r="I25" s="23"/>
       <c r="J25" s="23"/>
       <c r="K25" s="23"/>
-      <c r="BK25" s="1"/>
+      <c r="L25" t="s">
+        <v>240</v>
+      </c>
+      <c r="M25" t="s">
+        <v>202</v>
+      </c>
+      <c r="N25" t="s">
+        <v>203</v>
+      </c>
+      <c r="O25" t="s">
+        <v>204</v>
+      </c>
+      <c r="P25"/>
+      <c r="Q25"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25"/>
+      <c r="V25"/>
+      <c r="W25"/>
+      <c r="X25"/>
+      <c r="Y25"/>
+      <c r="Z25"/>
+      <c r="AA25"/>
+      <c r="AB25"/>
+      <c r="AC25"/>
+      <c r="AD25"/>
+      <c r="AE25"/>
+      <c r="AF25"/>
+      <c r="AG25"/>
+      <c r="AH25"/>
+      <c r="AI25"/>
+      <c r="AJ25"/>
+      <c r="AK25"/>
+      <c r="AL25"/>
+      <c r="AM25"/>
+      <c r="AN25"/>
+      <c r="AO25"/>
+      <c r="AP25"/>
+      <c r="AQ25"/>
+      <c r="AR25"/>
+      <c r="AS25"/>
+      <c r="AT25"/>
+      <c r="AU25"/>
+      <c r="AV25"/>
+      <c r="AW25"/>
+      <c r="AX25"/>
+      <c r="AY25"/>
+      <c r="AZ25"/>
+      <c r="BA25"/>
+      <c r="BB25"/>
+      <c r="BC25"/>
+      <c r="BD25"/>
+      <c r="BE25"/>
+      <c r="BF25"/>
+      <c r="BG25"/>
+      <c r="BH25"/>
+      <c r="BI25"/>
+      <c r="BJ25"/>
+      <c r="BK25" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="26">
-      <c r="H26" s="23"/>
+      <c r="A26" t="s">
+        <v>241</v>
+      </c>
+      <c r="B26" t="s">
+        <v>197</v>
+      </c>
+      <c r="C26" t="s">
+        <v>198</v>
+      </c>
+      <c r="D26" t="s">
+        <v>199</v>
+      </c>
+      <c r="E26" t="s">
+        <v>200</v>
+      </c>
+      <c r="F26" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G26"/>
+      <c r="H26" s="23" t="n">
+        <v>55.9</v>
+      </c>
       <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="BK26" s="1"/>
+      <c r="J26" s="23" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="K26" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="L26" t="s">
+        <v>242</v>
+      </c>
+      <c r="M26" t="s">
+        <v>202</v>
+      </c>
+      <c r="N26" t="s">
+        <v>203</v>
+      </c>
+      <c r="O26" t="s">
+        <v>204</v>
+      </c>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
+      <c r="W26"/>
+      <c r="X26"/>
+      <c r="Y26"/>
+      <c r="Z26"/>
+      <c r="AA26"/>
+      <c r="AB26"/>
+      <c r="AC26"/>
+      <c r="AD26"/>
+      <c r="AE26"/>
+      <c r="AF26"/>
+      <c r="AG26"/>
+      <c r="AH26"/>
+      <c r="AI26"/>
+      <c r="AJ26"/>
+      <c r="AK26"/>
+      <c r="AL26"/>
+      <c r="AM26"/>
+      <c r="AN26"/>
+      <c r="AO26"/>
+      <c r="AP26"/>
+      <c r="AQ26"/>
+      <c r="AR26"/>
+      <c r="AS26"/>
+      <c r="AT26"/>
+      <c r="AU26"/>
+      <c r="AV26"/>
+      <c r="AW26"/>
+      <c r="AX26"/>
+      <c r="AY26"/>
+      <c r="AZ26"/>
+      <c r="BA26"/>
+      <c r="BB26"/>
+      <c r="BC26"/>
+      <c r="BD26"/>
+      <c r="BE26"/>
+      <c r="BF26"/>
+      <c r="BG26"/>
+      <c r="BH26"/>
+      <c r="BI26"/>
+      <c r="BJ26"/>
+      <c r="BK26" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="27">
-      <c r="H27" s="23"/>
+      <c r="A27" t="s">
+        <v>243</v>
+      </c>
+      <c r="B27" t="s">
+        <v>197</v>
+      </c>
+      <c r="C27" t="s">
+        <v>198</v>
+      </c>
+      <c r="D27" t="s">
+        <v>199</v>
+      </c>
+      <c r="E27" t="s">
+        <v>200</v>
+      </c>
+      <c r="F27" t="n">
+        <v>44.35</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-108.39</v>
+      </c>
+      <c r="H27" s="23" t="n">
+        <v>55.6</v>
+      </c>
       <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="BK27" s="1"/>
+      <c r="J27" s="23" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="K27" s="23" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="L27" t="s">
+        <v>244</v>
+      </c>
+      <c r="M27" t="s">
+        <v>202</v>
+      </c>
+      <c r="N27" t="s">
+        <v>203</v>
+      </c>
+      <c r="O27" t="s">
+        <v>204</v>
+      </c>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27"/>
+      <c r="V27"/>
+      <c r="W27"/>
+      <c r="X27"/>
+      <c r="Y27"/>
+      <c r="Z27"/>
+      <c r="AA27"/>
+      <c r="AB27"/>
+      <c r="AC27"/>
+      <c r="AD27"/>
+      <c r="AE27"/>
+      <c r="AF27"/>
+      <c r="AG27"/>
+      <c r="AH27"/>
+      <c r="AI27"/>
+      <c r="AJ27"/>
+      <c r="AK27"/>
+      <c r="AL27"/>
+      <c r="AM27"/>
+      <c r="AN27"/>
+      <c r="AO27"/>
+      <c r="AP27"/>
+      <c r="AQ27"/>
+      <c r="AR27"/>
+      <c r="AS27"/>
+      <c r="AT27"/>
+      <c r="AU27"/>
+      <c r="AV27"/>
+      <c r="AW27"/>
+      <c r="AX27"/>
+      <c r="AY27"/>
+      <c r="AZ27"/>
+      <c r="BA27"/>
+      <c r="BB27"/>
+      <c r="BC27"/>
+      <c r="BD27"/>
+      <c r="BE27"/>
+      <c r="BF27"/>
+      <c r="BG27"/>
+      <c r="BH27"/>
+      <c r="BI27"/>
+      <c r="BJ27"/>
+      <c r="BK27" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="28">
-      <c r="H28" s="23"/>
+      <c r="A28" t="s">
+        <v>245</v>
+      </c>
+      <c r="B28" t="s">
+        <v>197</v>
+      </c>
+      <c r="C28" t="s">
+        <v>198</v>
+      </c>
+      <c r="D28" t="s">
+        <v>199</v>
+      </c>
+      <c r="E28" t="s">
+        <v>200</v>
+      </c>
+      <c r="F28" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-108.13</v>
+      </c>
+      <c r="H28" s="23" t="n">
+        <v>54.7</v>
+      </c>
       <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="BK28" s="1"/>
+      <c r="J28" s="23" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="K28" s="23" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="L28" t="s">
+        <v>246</v>
+      </c>
+      <c r="M28" t="s">
+        <v>202</v>
+      </c>
+      <c r="N28" t="s">
+        <v>203</v>
+      </c>
+      <c r="O28" t="s">
+        <v>204</v>
+      </c>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28"/>
+      <c r="AH28"/>
+      <c r="AI28"/>
+      <c r="AJ28"/>
+      <c r="AK28"/>
+      <c r="AL28"/>
+      <c r="AM28"/>
+      <c r="AN28"/>
+      <c r="AO28"/>
+      <c r="AP28"/>
+      <c r="AQ28"/>
+      <c r="AR28"/>
+      <c r="AS28"/>
+      <c r="AT28"/>
+      <c r="AU28"/>
+      <c r="AV28"/>
+      <c r="AW28"/>
+      <c r="AX28"/>
+      <c r="AY28"/>
+      <c r="AZ28"/>
+      <c r="BA28"/>
+      <c r="BB28"/>
+      <c r="BC28"/>
+      <c r="BD28"/>
+      <c r="BE28"/>
+      <c r="BF28"/>
+      <c r="BG28"/>
+      <c r="BH28"/>
+      <c r="BI28"/>
+      <c r="BJ28"/>
+      <c r="BK28" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="29">
-      <c r="H29" s="23"/>
+      <c r="A29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B29" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" t="s">
+        <v>198</v>
+      </c>
+      <c r="D29" t="s">
+        <v>199</v>
+      </c>
+      <c r="E29" t="s">
+        <v>200</v>
+      </c>
+      <c r="F29" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="G29"/>
+      <c r="H29" s="23" t="n">
+        <v>54.3</v>
+      </c>
       <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="23"/>
-      <c r="BK29" s="1"/>
+      <c r="J29" s="23" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="K29" s="23" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="L29" t="s">
+        <v>248</v>
+      </c>
+      <c r="M29" t="s">
+        <v>202</v>
+      </c>
+      <c r="N29" t="s">
+        <v>203</v>
+      </c>
+      <c r="O29" t="s">
+        <v>204</v>
+      </c>
+      <c r="P29"/>
+      <c r="Q29"/>
+      <c r="R29"/>
+      <c r="S29"/>
+      <c r="T29"/>
+      <c r="U29"/>
+      <c r="V29"/>
+      <c r="W29"/>
+      <c r="X29"/>
+      <c r="Y29"/>
+      <c r="Z29"/>
+      <c r="AA29"/>
+      <c r="AB29"/>
+      <c r="AC29"/>
+      <c r="AD29"/>
+      <c r="AE29"/>
+      <c r="AF29"/>
+      <c r="AG29"/>
+      <c r="AH29"/>
+      <c r="AI29"/>
+      <c r="AJ29"/>
+      <c r="AK29"/>
+      <c r="AL29"/>
+      <c r="AM29"/>
+      <c r="AN29"/>
+      <c r="AO29"/>
+      <c r="AP29"/>
+      <c r="AQ29"/>
+      <c r="AR29"/>
+      <c r="AS29"/>
+      <c r="AT29"/>
+      <c r="AU29"/>
+      <c r="AV29"/>
+      <c r="AW29"/>
+      <c r="AX29"/>
+      <c r="AY29"/>
+      <c r="AZ29"/>
+      <c r="BA29"/>
+      <c r="BB29"/>
+      <c r="BC29"/>
+      <c r="BD29"/>
+      <c r="BE29"/>
+      <c r="BF29"/>
+      <c r="BG29"/>
+      <c r="BH29"/>
+      <c r="BI29"/>
+      <c r="BJ29"/>
+      <c r="BK29" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="30">
-      <c r="H30" s="23"/>
+      <c r="A30" t="s">
+        <v>249</v>
+      </c>
+      <c r="B30" t="s">
+        <v>197</v>
+      </c>
+      <c r="C30" t="s">
+        <v>198</v>
+      </c>
+      <c r="D30" t="s">
+        <v>199</v>
+      </c>
+      <c r="E30" t="s">
+        <v>200</v>
+      </c>
+      <c r="F30" t="n">
+        <v>44.35</v>
+      </c>
+      <c r="G30"/>
+      <c r="H30" s="23" t="n">
+        <v>54.2</v>
+      </c>
       <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="23"/>
-      <c r="BK30" s="1"/>
+      <c r="J30" s="23" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="K30" s="23" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="L30" t="s">
+        <v>250</v>
+      </c>
+      <c r="M30" t="s">
+        <v>202</v>
+      </c>
+      <c r="N30" t="s">
+        <v>203</v>
+      </c>
+      <c r="O30" t="s">
+        <v>204</v>
+      </c>
+      <c r="P30"/>
+      <c r="Q30"/>
+      <c r="R30"/>
+      <c r="S30"/>
+      <c r="T30"/>
+      <c r="U30"/>
+      <c r="V30"/>
+      <c r="W30"/>
+      <c r="X30"/>
+      <c r="Y30"/>
+      <c r="Z30"/>
+      <c r="AA30"/>
+      <c r="AB30"/>
+      <c r="AC30"/>
+      <c r="AD30"/>
+      <c r="AE30"/>
+      <c r="AF30"/>
+      <c r="AG30"/>
+      <c r="AH30"/>
+      <c r="AI30"/>
+      <c r="AJ30"/>
+      <c r="AK30"/>
+      <c r="AL30"/>
+      <c r="AM30"/>
+      <c r="AN30"/>
+      <c r="AO30"/>
+      <c r="AP30"/>
+      <c r="AQ30"/>
+      <c r="AR30"/>
+      <c r="AS30"/>
+      <c r="AT30"/>
+      <c r="AU30"/>
+      <c r="AV30"/>
+      <c r="AW30"/>
+      <c r="AX30"/>
+      <c r="AY30"/>
+      <c r="AZ30"/>
+      <c r="BA30"/>
+      <c r="BB30"/>
+      <c r="BC30"/>
+      <c r="BD30"/>
+      <c r="BE30"/>
+      <c r="BF30"/>
+      <c r="BG30"/>
+      <c r="BH30"/>
+      <c r="BI30"/>
+      <c r="BJ30"/>
+      <c r="BK30" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="31">
-      <c r="H31" s="23"/>
+      <c r="A31" t="s">
+        <v>251</v>
+      </c>
+      <c r="B31" t="s">
+        <v>197</v>
+      </c>
+      <c r="C31" t="s">
+        <v>198</v>
+      </c>
+      <c r="D31" t="s">
+        <v>199</v>
+      </c>
+      <c r="E31" t="s">
+        <v>200</v>
+      </c>
+      <c r="F31" t="n">
+        <v>46.52</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-116.75</v>
+      </c>
+      <c r="H31" s="23" t="n">
+        <v>16.5</v>
+      </c>
       <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="BK31" s="1"/>
+      <c r="J31" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="K31" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="L31" t="s">
+        <v>252</v>
+      </c>
+      <c r="M31" t="s">
+        <v>202</v>
+      </c>
+      <c r="N31" t="s">
+        <v>203</v>
+      </c>
+      <c r="O31" t="s">
+        <v>204</v>
+      </c>
+      <c r="P31"/>
+      <c r="Q31"/>
+      <c r="R31"/>
+      <c r="S31"/>
+      <c r="T31"/>
+      <c r="U31"/>
+      <c r="V31"/>
+      <c r="W31"/>
+      <c r="X31"/>
+      <c r="Y31"/>
+      <c r="Z31"/>
+      <c r="AA31"/>
+      <c r="AB31"/>
+      <c r="AC31"/>
+      <c r="AD31"/>
+      <c r="AE31"/>
+      <c r="AF31"/>
+      <c r="AG31"/>
+      <c r="AH31"/>
+      <c r="AI31"/>
+      <c r="AJ31"/>
+      <c r="AK31"/>
+      <c r="AL31"/>
+      <c r="AM31"/>
+      <c r="AN31"/>
+      <c r="AO31"/>
+      <c r="AP31"/>
+      <c r="AQ31"/>
+      <c r="AR31"/>
+      <c r="AS31"/>
+      <c r="AT31"/>
+      <c r="AU31"/>
+      <c r="AV31"/>
+      <c r="AW31"/>
+      <c r="AX31"/>
+      <c r="AY31"/>
+      <c r="AZ31"/>
+      <c r="BA31"/>
+      <c r="BB31"/>
+      <c r="BC31"/>
+      <c r="BD31"/>
+      <c r="BE31"/>
+      <c r="BF31"/>
+      <c r="BG31"/>
+      <c r="BH31"/>
+      <c r="BI31"/>
+      <c r="BJ31"/>
+      <c r="BK31" s="1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="32">
-      <c r="H32" s="23"/>
+      <c r="A32" t="s">
+        <v>253</v>
+      </c>
+      <c r="B32" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" t="s">
+        <v>198</v>
+      </c>
+      <c r="D32" t="s">
+        <v>199</v>
+      </c>
+      <c r="E32" t="s">
+        <v>200</v>
+      </c>
+      <c r="F32" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-116.27</v>
+      </c>
+      <c r="H32" s="23" t="n">
+        <v>15.78</v>
+      </c>
       <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="BK32" s="1"/>
+      <c r="J32" s="23" t="n">
+        <v>15.741</v>
+      </c>
+      <c r="K32" s="23" t="n">
+        <v>15.819</v>
+      </c>
+      <c r="L32" t="s">
+        <v>254</v>
+      </c>
+      <c r="M32" t="s">
+        <v>255</v>
+      </c>
+      <c r="N32" t="s">
+        <v>256</v>
+      </c>
+      <c r="O32" t="s">
+        <v>257</v>
+      </c>
+      <c r="P32"/>
+      <c r="Q32"/>
+      <c r="R32"/>
+      <c r="S32"/>
+      <c r="T32"/>
+      <c r="U32"/>
+      <c r="V32"/>
+      <c r="W32"/>
+      <c r="X32"/>
+      <c r="Y32"/>
+      <c r="Z32"/>
+      <c r="AA32"/>
+      <c r="AB32"/>
+      <c r="AC32"/>
+      <c r="AD32"/>
+      <c r="AE32"/>
+      <c r="AF32"/>
+      <c r="AG32"/>
+      <c r="AH32"/>
+      <c r="AI32"/>
+      <c r="AJ32"/>
+      <c r="AK32"/>
+      <c r="AL32"/>
+      <c r="AM32"/>
+      <c r="AN32"/>
+      <c r="AO32"/>
+      <c r="AP32"/>
+      <c r="AQ32"/>
+      <c r="AR32"/>
+      <c r="AS32"/>
+      <c r="AT32"/>
+      <c r="AU32"/>
+      <c r="AV32"/>
+      <c r="AW32"/>
+      <c r="AX32"/>
+      <c r="AY32"/>
+      <c r="AZ32"/>
+      <c r="BA32"/>
+      <c r="BB32"/>
+      <c r="BC32"/>
+      <c r="BD32"/>
+      <c r="BE32"/>
+      <c r="BF32"/>
+      <c r="BG32"/>
+      <c r="BH32"/>
+      <c r="BI32"/>
+      <c r="BJ32"/>
+      <c r="BK32" s="1" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="33">
-      <c r="H33" s="23"/>
+      <c r="A33" t="s">
+        <v>259</v>
+      </c>
+      <c r="B33" t="s">
+        <v>197</v>
+      </c>
+      <c r="C33" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" t="s">
+        <v>199</v>
+      </c>
+      <c r="E33" t="s">
+        <v>200</v>
+      </c>
+      <c r="F33" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-116.27</v>
+      </c>
+      <c r="H33" s="23" t="n">
+        <v>15.78</v>
+      </c>
       <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="23"/>
-      <c r="BK33" s="1"/>
+      <c r="J33" s="23" t="n">
+        <v>15.741</v>
+      </c>
+      <c r="K33" s="23" t="n">
+        <v>15.819</v>
+      </c>
+      <c r="L33" t="s">
+        <v>254</v>
+      </c>
+      <c r="M33" t="s">
+        <v>255</v>
+      </c>
+      <c r="N33" t="s">
+        <v>256</v>
+      </c>
+      <c r="O33" t="s">
+        <v>257</v>
+      </c>
+      <c r="P33"/>
+      <c r="Q33"/>
+      <c r="R33"/>
+      <c r="S33"/>
+      <c r="T33"/>
+      <c r="U33"/>
+      <c r="V33"/>
+      <c r="W33"/>
+      <c r="X33"/>
+      <c r="Y33"/>
+      <c r="Z33"/>
+      <c r="AA33"/>
+      <c r="AB33"/>
+      <c r="AC33"/>
+      <c r="AD33"/>
+      <c r="AE33"/>
+      <c r="AF33"/>
+      <c r="AG33"/>
+      <c r="AH33"/>
+      <c r="AI33"/>
+      <c r="AJ33"/>
+      <c r="AK33"/>
+      <c r="AL33"/>
+      <c r="AM33"/>
+      <c r="AN33"/>
+      <c r="AO33"/>
+      <c r="AP33"/>
+      <c r="AQ33"/>
+      <c r="AR33"/>
+      <c r="AS33"/>
+      <c r="AT33"/>
+      <c r="AU33"/>
+      <c r="AV33"/>
+      <c r="AW33"/>
+      <c r="AX33"/>
+      <c r="AY33"/>
+      <c r="AZ33"/>
+      <c r="BA33"/>
+      <c r="BB33"/>
+      <c r="BC33"/>
+      <c r="BD33"/>
+      <c r="BE33"/>
+      <c r="BF33"/>
+      <c r="BG33"/>
+      <c r="BH33"/>
+      <c r="BI33"/>
+      <c r="BJ33"/>
+      <c r="BK33" s="1" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="34">
-      <c r="H34" s="23"/>
+      <c r="A34" t="s">
+        <v>260</v>
+      </c>
+      <c r="B34" t="s">
+        <v>197</v>
+      </c>
+      <c r="C34" t="s">
+        <v>198</v>
+      </c>
+      <c r="D34" t="s">
+        <v>199</v>
+      </c>
+      <c r="E34" t="s">
+        <v>200</v>
+      </c>
+      <c r="F34" t="n">
+        <v>47.03</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-116.34</v>
+      </c>
+      <c r="H34" s="23" t="n">
+        <v>15.78</v>
+      </c>
       <c r="I34" s="23"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="23"/>
-      <c r="BK34" s="1"/>
+      <c r="J34" s="23" t="n">
+        <v>15.741</v>
+      </c>
+      <c r="K34" s="23" t="n">
+        <v>15.819</v>
+      </c>
+      <c r="L34" t="s">
+        <v>261</v>
+      </c>
+      <c r="M34" t="s">
+        <v>255</v>
+      </c>
+      <c r="N34" t="s">
+        <v>256</v>
+      </c>
+      <c r="O34" t="s">
+        <v>257</v>
+      </c>
+      <c r="P34"/>
+      <c r="Q34"/>
+      <c r="R34"/>
+      <c r="S34"/>
+      <c r="T34"/>
+      <c r="U34"/>
+      <c r="V34"/>
+      <c r="W34"/>
+      <c r="X34"/>
+      <c r="Y34"/>
+      <c r="Z34"/>
+      <c r="AA34"/>
+      <c r="AB34"/>
+      <c r="AC34"/>
+      <c r="AD34"/>
+      <c r="AE34"/>
+      <c r="AF34"/>
+      <c r="AG34"/>
+      <c r="AH34"/>
+      <c r="AI34"/>
+      <c r="AJ34"/>
+      <c r="AK34"/>
+      <c r="AL34"/>
+      <c r="AM34"/>
+      <c r="AN34"/>
+      <c r="AO34"/>
+      <c r="AP34"/>
+      <c r="AQ34"/>
+      <c r="AR34"/>
+      <c r="AS34"/>
+      <c r="AT34"/>
+      <c r="AU34"/>
+      <c r="AV34"/>
+      <c r="AW34"/>
+      <c r="AX34"/>
+      <c r="AY34"/>
+      <c r="AZ34"/>
+      <c r="BA34"/>
+      <c r="BB34"/>
+      <c r="BC34"/>
+      <c r="BD34"/>
+      <c r="BE34"/>
+      <c r="BF34"/>
+      <c r="BG34"/>
+      <c r="BH34"/>
+      <c r="BI34"/>
+      <c r="BJ34"/>
+      <c r="BK34" s="1" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="35">
       <c r="H35" s="23"/>

</xml_diff>